<commit_message>
Add current 216-issue scoring table while preserving validation snapshot
</commit_message>
<xml_diff>
--- a/2_Exercise_Materials/scoring_tables/Job_Exercise_Scoring_Table_Main.xlsx
+++ b/2_Exercise_Materials/scoring_tables/Job_Exercise_Scoring_Table_Main.xlsx
@@ -2,10 +2,27 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring table" sheetId="1" r:id="R8aeea17e61f14f5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring logic" sheetId="2" r:id="Rdd369c99fd0e4c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring table" sheetId="1" r:id="R4edb0b64de5b4056"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring logic" sheetId="2" r:id="R73f0498dc571411c"/>
   </x:sheets>
 </x:workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:authors>
+    <x:author/>
+  </x:authors>
+  <x:commentList>
+    <x:comment ref="A217" authorId="0">
+      <x:text>
+        <x:r>
+          <x:t>This issue was added after the October 27, 2026 pilot data collection, when we realized that the scorer could not assign a score to it.</x:t>
+        </x:r>
+      </x:text>
+    </x:comment>
+  </x:commentList>
+</x:comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -101,8 +118,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="JobScoringtable" displayName="JobScoringtable" ref="A1:E637" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:E637"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="JobScoringtable" displayName="JobScoringtable" ref="A1:E639" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:E639"/>
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Issue"/>
     <x:tableColumn id="2" name="Discrete/continuous"/>
@@ -115,8 +132,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="JobScoringlogic" displayName="JobScoringlogic" ref="A1:D216" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:D216"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="JobScoringlogic" displayName="JobScoringlogic" ref="A1:D217" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:D217"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Issue"/>
     <x:tableColumn id="2" name="What it covers"/>
@@ -11158,10 +11175,44 @@
         <x:v>-1</x:v>
       </x:c>
     </x:row>
+    <x:row r="638" ht="31.5" customHeight="1">
+      <x:c r="A638" s="5" t="str">
+        <x:v>Workplace Coffee</x:v>
+      </x:c>
+      <x:c r="B638" s="4" t="str">
+        <x:v>Discrete</x:v>
+      </x:c>
+      <x:c r="C638" s="4" t="str">
+        <x:v>Free coffee provided</x:v>
+      </x:c>
+      <x:c r="D638" s="9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E638" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="639" ht="31.5" customHeight="1">
+      <x:c r="A639" s="5" t="str">
+        <x:v>Workplace Coffee</x:v>
+      </x:c>
+      <x:c r="B639" s="4" t="str">
+        <x:v>Discrete</x:v>
+      </x:c>
+      <x:c r="C639" s="4" t="str">
+        <x:v>No free coffee provided</x:v>
+      </x:c>
+      <x:c r="D639" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E639" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa521de266ad480b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c8c428c58344bdc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14200,10 +14251,25 @@
         <x:v>+1 for Attend the monthly sales planning meeting; 0 for No access to planning meetings; −1 for Attend all management meetings. The company wants coordination and protecting management time and confidential information.</x:v>
       </x:c>
     </x:row>
+    <x:row r="217" ht="84" customHeight="1">
+      <x:c r="A217" s="5" t="str">
+        <x:v>Workplace Coffee</x:v>
+      </x:c>
+      <x:c r="B217" s="4" t="str">
+        <x:v>Whether the company provides coffee free of charge in the workplace.</x:v>
+      </x:c>
+      <x:c r="C217" s="4" t="str">
+        <x:v>+1 when free workplace coffee is provided; 0 otherwise. It is a small daily benefit that makes working in the office more comfortable.</x:v>
+      </x:c>
+      <x:c r="D217" s="4" t="str">
+        <x:v>0 whether coffee is provided or not. This small workplace amenity is treated as neutral to the hiring decision.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0f829e46bea46fd"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d8190a4575d4027"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ee6d1a5bb8b4f0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>